<commit_message>
few updates in experience and skills
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Basic Info"/>
@@ -35,34 +35,34 @@
     <t>Info</t>
   </si>
   <si>
-    <t>Thapar Acm Student Chapter</t>
-  </si>
-  <si>
-    <t>Event Management</t>
-  </si>
-  <si>
-    <t>static/acm.png</t>
-  </si>
-  <si>
-    <t>Oct 2020 - July 2022</t>
-  </si>
-  <si>
-    <t>Orchestrated the highly successful Eclipse event, integrating a Hackathon, Competitive Programming, and Designing; collaborated with the Tech team to design a seamless registration portal resulting in 500+ participants</t>
-  </si>
-  <si>
-    <t>National Service Scheme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Member </t>
-  </si>
-  <si>
-    <t>static/nss.png</t>
-  </si>
-  <si>
-    <t>Oct 2021 - Nov 2022</t>
-  </si>
-  <si>
-    <t>Collected old winter clothes from students and faculty and distributed to needy people.</t>
+    <t>Capgemini India Private Limited&amp;#10;</t>
+  </si>
+  <si>
+    <t>Senior Analyst</t>
+  </si>
+  <si>
+    <t>static/capg.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> November 2024 - Present</t>
+  </si>
+  <si>
+    <t>• Worked on Snowflake across DEV, QAT, and PROD for data modeling, performance tuning, and validation, improving&amp;#10;data handling efficiency by 25%.&amp;#10;• Automated end-to-end data validation using Python and SQL, reducing manual QA effort by 60%.&amp;#10;• Built a Python-based metadata monitoring framework using dynamic threshold checks and real-time email alerts,&amp;#10;reducing error detection time by 40%.&amp;#10;• Leveraged Cosine Similarity and SLM models for automated data mapping, improving mapping accuracy by 30% and&amp;#10;generating insights for Excel-based reports.&amp;#10;• Implemented Snowflake Stages &amp; Snowpipes for Disaster Recovery (US-East-2), enabling automatic data synchronization&amp;#10;and backup.&amp;#10;• Used Jenkins + UDeploy for automated deployment of Snowflake objects and Python updates, reducing deployment time&amp;#10;and avoiding manual errors.&amp;#10;• Worked on Informatica IDMC for da</t>
+  </si>
+  <si>
+    <t>Alpha Net Solutions</t>
+  </si>
+  <si>
+    <t>Development Intern</t>
+  </si>
+  <si>
+    <t>static/alphanet.png</t>
+  </si>
+  <si>
+    <t>January 2024 - July 2024</t>
+  </si>
+  <si>
+    <t>• Blog Portal - Engineered and crafted the frontend using pure HTML, CSS, and JavaScript, ensuring a responsive and&amp;#10;user-friendly interface with media queries, resulting in a 40% increase in user satisfaction.&amp;#10;• Designed and implemented an intuitive admin dashboard to facilitate CRUD operations, enabling administrators to&amp;#10;efficiently manage blog content and user accounts, thereby reducing content update time by 50%.&amp;#10;• Crafted the backend using PHP and MySQL, leveraging phpmyadmin for database management.&amp;#10;• Added a search feature to enable users to find specific blog posts quickly.</t>
   </si>
   <si>
     <t>Institute</t>
@@ -161,46 +161,46 @@
     <t>static/python.png</t>
   </si>
   <si>
-    <t>3 yrs</t>
-  </si>
-  <si>
-    <t>Web Development</t>
-  </si>
-  <si>
-    <t>static/wd.webp</t>
-  </si>
-  <si>
-    <t>2 yrs</t>
-  </si>
-  <si>
-    <t>Machine Learning</t>
-  </si>
-  <si>
-    <t>static/ml.png</t>
-  </si>
-  <si>
-    <t>Cloud Computing</t>
-  </si>
-  <si>
-    <t>static/cloud.png</t>
-  </si>
-  <si>
-    <t>1 yrs</t>
-  </si>
-  <si>
-    <t>Blockchain Technology</t>
-  </si>
-  <si>
-    <t>static/block.webp</t>
-  </si>
-  <si>
-    <t>Data Science</t>
-  </si>
-  <si>
-    <t>static/ds.png</t>
-  </si>
-  <si>
-    <t/>
+    <t>2 years</t>
+  </si>
+  <si>
+    <t>SQL</t>
+  </si>
+  <si>
+    <t>static/sql.png</t>
+  </si>
+  <si>
+    <t>Snowflake</t>
+  </si>
+  <si>
+    <t>static/snowflake.png</t>
+  </si>
+  <si>
+    <t>1 year</t>
+  </si>
+  <si>
+    <t>Jenkins</t>
+  </si>
+  <si>
+    <t>static/jenkins.jpeg</t>
+  </si>
+  <si>
+    <t>UDeploy</t>
+  </si>
+  <si>
+    <t>static/udeploy.png</t>
+  </si>
+  <si>
+    <t>AutoSys</t>
+  </si>
+  <si>
+    <t>static/autosys.jpg</t>
+  </si>
+  <si>
+    <t>IDMC</t>
+  </si>
+  <si>
+    <t>static/idmc.jpg</t>
   </si>
   <si>
     <t>Column</t>
@@ -215,10 +215,10 @@
     <t>Pranshu Verma</t>
   </si>
   <si>
-    <t>Aspiring Python Developer</t>
-  </si>
-  <si>
-    <t>I am also a final year student at Thapar Institute of Engineering and Technology, pursuing a Bachelor of Technology in Electronics and Computer Engineering. I have a keen interest in problem-solving and web development, and I constantly seek to learn new things and improve my skills. I have completed several online courses and certifications in Python, ML, and SQL, and I have applied my knowledge to develop ML models and databases for various academic and personal projects. I am motivated by the challenges and opportunities that web development and ML offer, and I aspire to become a full-stack developer in the future.</t>
+    <t>Data Engineer / Data Analyst</t>
+  </si>
+  <si>
+    <t>Data Engineer with experience in Snowflake, Python automation, cloud data warehousing, data validation frameworks, and CI/CD deployment. Skilled in SQL, Informatica IDMC, automated reporting, and metadata-based monitoring. Strong analytical mindset with hands-on experience in data processing, pipeline development, and statistical analysis. Looking for roles in Data Engineering / Data Analytics / Marketing Analytics</t>
   </si>
   <si>
     <t>Photo</t>
@@ -254,7 +254,7 @@
     <t>Resume Link</t>
   </si>
   <si>
-    <t>https://drive.google.com/file/d/1CDZyw8KESQkU5HtPn51jJbVUVx_Uq_cT/view?usp=drive_link</t>
+    <t>https://drive.google.com/file/d/1O3QVWbLLfMPFz8D-rNotwVtLZ74WWiCx/view?usp=sharing</t>
   </si>
   <si>
     <t>Note</t>
@@ -285,13 +285,13 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -333,42 +333,42 @@
   <cellXfs count="14">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
   </cellXfs>
@@ -676,113 +676,113 @@
   <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="18.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="43.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="7" width="18.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="43.71928571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>62</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="13" t="s">
         <v>64</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="13" t="s">
         <v>65</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="13" t="s">
         <v>66</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="13" t="s">
         <v>68</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="13" t="s">
         <v>70</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="13" t="s">
         <v>72</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="13" t="s">
         <v>74</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="13" t="s">
         <v>76</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="13" t="s">
         <v>78</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="2"/>
+      <c r="B14" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="B15" s="2"/>
+      <c r="B15" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -797,97 +797,97 @@
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="15.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="23.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="9.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="7" width="15.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="23.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="9.862142857142858" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="13" t="s">
         <v>47</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="13" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>50</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="13" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="13" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="13" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>55</v>
+      <c r="C7" s="13" t="s">
+        <v>52</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>60</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -903,71 +903,71 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="20.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="12.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="11.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="3" width="102.29071428571429" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="7" width="20.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="12.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="11.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="102.29071428571429" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="13" t="s">
         <v>38</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="13" t="s">
         <v>42</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -990,86 +990,86 @@
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75" customFormat="1" s="5">
-      <c r="A2" s="6" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75" customFormat="1" s="3">
+      <c r="A2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75" customFormat="1" s="5">
-      <c r="A3" s="6" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75" customFormat="1" s="3">
+      <c r="A3" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="8" t="s">
         <v>27</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75" customFormat="1" s="5">
-      <c r="A5" s="6"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75" customFormat="1" s="5">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75" customFormat="1" s="3">
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75" customFormat="1" s="3">
       <c r="A6" s="10"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1084,61 +1084,61 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="15.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="15.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="3" width="17.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="15.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="15.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="17.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="1008.75" customFormat="1" s="3">
+      <c r="A2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="666" customFormat="1" s="3">
+      <c r="A3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="4" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>